<commit_message>
facilitating pre-selection of optimal run configuration; adding progress messages to visualisation script
</commit_message>
<xml_diff>
--- a/2_REVUB_control_file/control_file.xlsx
+++ b/2_REVUB_control_file/control_file.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/REVUB code repo/2_REVUB_control_files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/REVUB code repo/2_REVUB_control_file/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1196" documentId="13_ncr:1_{3E75B3F6-DB26-4BD5-A9C7-B5D5CA9FF346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58F92CB1-02DC-4781-8FD9-8F2F2A5BC059}"/>
+  <xr:revisionPtr revIDLastSave="1204" documentId="13_ncr:1_{3E75B3F6-DB26-4BD5-A9C7-B5D5CA9FF346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5798BDAE-4F46-4712-9867-F816114537D9}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="735" xr2:uid="{B27AEA38-A928-4B6A-AF9B-7A28216807AA}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="213">
   <si>
     <t>Hydropower plants</t>
   </si>
@@ -1554,6 +1554,60 @@
   </si>
   <si>
     <t>tables_on_multiple</t>
+  </si>
+  <si>
+    <t>f_init_BAL_opt</t>
+  </si>
+  <si>
+    <t>f_init_STOR_opt</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[only use if already known from previous run]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The optimal value in the range of the ELCC for STOR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[only use if already known from previous run]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The optimal value in the range of the ELCC for BAL</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2163,7 +2217,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10D23870-37A0-4EFA-BF75-9E0BBC5C39B4}">
-  <dimension ref="A1:M61"/>
+  <dimension ref="A1:M63"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.81640625" style="5" customWidth="1"/>
@@ -2560,96 +2614,112 @@
         <v>92</v>
       </c>
     </row>
-    <row r="50" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
-      <c r="A50" s="9" t="s">
+    <row r="50" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A50" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
+      <c r="A51" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="B50" s="7"/>
-    </row>
-    <row r="51" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B51" s="19" t="s">
-        <v>95</v>
-      </c>
+      <c r="B51" s="7"/>
     </row>
     <row r="52" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
+      </c>
+      <c r="B52" s="19" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="53" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="B53" s="19" t="s">
-        <v>99</v>
+        <v>96</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="54" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B54" s="19" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="55" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
+      </c>
+      <c r="B55" s="19" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="56" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B57" s="1" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="57" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
-      <c r="A57" s="9" t="s">
+    <row r="58" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
+      <c r="A58" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="B57" s="7"/>
-    </row>
-    <row r="58" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A58" s="5" t="s">
+      <c r="B58" s="7"/>
+    </row>
+    <row r="59" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A59" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B59" s="1" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="59" spans="1:2" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A59" s="5" t="s">
+    <row r="60" spans="1:2" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A60" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B60" s="1" t="s">
         <v>110</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A60" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="61" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A62" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B62" s="1" t="s">
         <v>114</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A63" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>